<commit_message>
Agent Levels Fix, Statement Processing File Fixes, Edit Product Fixes
</commit_message>
<xml_diff>
--- a/TestFiles-prod-sanity/StatementProcessing/[MLB NEW]HappyFlowChangeCheckRunDate.xlsx
+++ b/TestFiles-prod-sanity/StatementProcessing/[MLB NEW]HappyFlowChangeCheckRunDate.xlsx
@@ -76,13 +76,13 @@
     <t>Premium</t>
   </si>
   <si>
-    <t>Agent</t>
-  </si>
-  <si>
-    <t>test-DevaTest</t>
-  </si>
-  <si>
-    <t>0987654321</t>
+    <t>Test</t>
+  </si>
+  <si>
+    <t>test-AgentX</t>
+  </si>
+  <si>
+    <t>600011</t>
   </si>
   <si>
     <t>232 E KING ST2 , ,, MALVERN, PA, 19355</t>
@@ -91,7 +91,7 @@
     <t>Integrity Health, LLC</t>
   </si>
   <si>
-    <t>IANG12370001IL001</t>
+    <t>IANG12370001IL211</t>
   </si>
   <si>
     <t>ROBERTS, PIPPIN</t>
@@ -630,7 +630,7 @@
         <v>28</v>
       </c>
       <c r="Q2" s="9">
-        <v>46024</v>
+        <v>46053</v>
       </c>
       <c r="R2" s="4" t="s">
         <v>29</v>

</xml_diff>